<commit_message>
site build 2026-10-09 07:33
</commit_message>
<xml_diff>
--- a/models/sovereigns/Kuwait_Sovereign_Model.xlsx
+++ b/models/sovereigns/Kuwait_Sovereign_Model.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -660,11 +660,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>BIS WS_CBPOL monthly series (auto-filled; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -777,7 +773,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>22.3</v>
+        <v>2.9</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -786,12 +782,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>FY24/25</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>Search summary of debt law coverage (tier 4)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -801,7 +797,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+          <t>Gross government debt, press forecast path (about 12% by FY27/28); conflicts with repo WEO 22.3%, unresolved</t>
         </is>
       </c>
     </row>
@@ -829,7 +825,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>27.6</v>
+        <v>-18.5</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -838,24 +834,20 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>FY26/27 draft budget (KD 9.8bn / $31.9bn deficit over repo nominal GDP, derived)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>Arab News, Kuwait Times, TradeArabia; ratio derived in the adjudicated document</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+          <t>28-Feb-26</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -915,7 +907,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>26</v>
+        <v>18.8</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -924,12 +916,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>2025-Q2 to 2026-Q1 (4-quarter sum USD 32.54bn over repo nominal GDP, derived)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF BOP via repo data record; ratio derived in the adjudicated document</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -937,11 +929,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -994,7 +982,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1009,7 +997,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Gross official reserves incl. gold at national valuation, end-month (auto-filled; a run's sourced point replaces it unless older)</t>
+          <t>CBK gross reserves incl. gold (gold USD 0.103bn)</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1025,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>8.406000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1059,11 +1047,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1123,7 +1107,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>172.92</v>
+        <v>172.9</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1132,12 +1116,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026E</t>
+          <t>not stated in repo record</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>Repo data record database/sovereigns/kuwait.json (IMF WEO via repo)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1145,11 +1129,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1247,6 +1227,21 @@
           <t>fitch</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1254,11 +1249,31 @@
           <t>sp</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>21-Nov-25</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
           <t>moodys</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Stable</t>
         </is>
       </c>
     </row>

</xml_diff>